<commit_message>
feat: correct registration number for FRT 41 (DULHADEPUR) in migration script
</commit_message>
<xml_diff>
--- a/Vehicles.xlsx
+++ b/Vehicles.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\FRT-VMS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F35A120-8C25-412E-8118-F85A2B03BA9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B822EC9E-708B-4A28-A8E7-978C2E7D2DDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -753,13 +753,13 @@
     <t>UP78MN4595</t>
   </si>
   <si>
-    <t>UP78ST3092</t>
-  </si>
-  <si>
     <t>BHILWAL</t>
   </si>
   <si>
     <t>SIDHAUR</t>
+  </si>
+  <si>
+    <t>UP78FT3092</t>
   </si>
 </sst>
 </file>
@@ -2473,7 +2473,7 @@
         <v>104</v>
       </c>
       <c r="C26" s="96" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="D26" s="16" t="s">
         <v>105</v>
@@ -2579,7 +2579,7 @@
         <v>116</v>
       </c>
       <c r="C29" s="96" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="D29" s="16" t="s">
         <v>117</v>
@@ -2994,7 +2994,7 @@
         <v>161</v>
       </c>
       <c r="D42" s="95" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E42" s="23"/>
       <c r="F42" s="23"/>

</xml_diff>

<commit_message>
feat: add vendor mobile information to vehicle records and update related components
</commit_message>
<xml_diff>
--- a/Vehicles.xlsx
+++ b/Vehicles.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\FRT-VMS\vehicle-info\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\FRT-VMS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9875629E-669E-4B05-9D6C-5EB7FE43D207}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DDE2A4E-BCE1-4353-88CF-8C407E910832}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>